<commit_message>
relatorios mês junho sku
</commit_message>
<xml_diff>
--- a/saida_skus/SKU_UTD-028-CZ-ORGANIZADOR-TAMPA.xlsx
+++ b/saida_skus/SKU_UTD-028-CZ-ORGANIZADOR-TAMPA.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analise" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$85</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -33,11 +33,11 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00008000"/>
+      <color rgb="00D93025"/>
     </font>
     <font>
       <b val="1"/>
-      <color rgb="00D93025"/>
+      <color rgb="00008000"/>
     </font>
   </fonts>
   <fills count="3">
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O64"/>
+  <dimension ref="A1:O85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -559,12 +559,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>23/06/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -598,11 +598,11 @@
         </is>
       </c>
       <c r="I2" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>▲ 100,0%</t>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
@@ -632,12 +632,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -665,17 +665,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+        <v>3</v>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>▼ 25,0%</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr">
@@ -705,12 +705,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -735,7 +735,7 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 35,00</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
@@ -744,7 +744,7 @@
         </is>
       </c>
       <c r="I4" s="2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
@@ -753,15 +753,15 @@
       </c>
       <c r="K4" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>25,0%</t>
         </is>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -778,12 +778,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>29/05/2026</t>
+          <t>19/06/2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -811,15 +811,15 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="3" t="inlineStr">
         <is>
           <t>▼ 100,0%</t>
         </is>
@@ -851,12 +851,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>29/05/2026</t>
+          <t>19/06/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>28/05/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -881,7 +881,7 @@
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>R$ 38,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
@@ -890,24 +890,24 @@
         </is>
       </c>
       <c r="I6" s="2" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>▲ 150,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
         <is>
-          <t>20,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>0,6%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -924,12 +924,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>28/05/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>17/06/2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -963,11 +963,11 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>▼ 50,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>▼ 75,0%</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
@@ -997,12 +997,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>17/06/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1038,7 +1038,7 @@
       <c r="I8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J8" s="3" t="inlineStr">
+      <c r="J8" s="4" t="inlineStr">
         <is>
           <t>▲ 300,0%</t>
         </is>
@@ -1070,12 +1070,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1111,9 +1111,9 @@
       <c r="I9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>▼ 50,0%</t>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>▼ 75,0%</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1143,12 +1143,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>14/06/2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1182,9 +1182,9 @@
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
         <is>
           <t>▲ 100,0%</t>
         </is>
@@ -1216,12 +1216,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>14/06/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1255,11 +1255,11 @@
         </is>
       </c>
       <c r="I11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>▼ 50,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>12/06/2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1332,7 +1332,7 @@
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1362,12 +1362,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>12/06/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1395,17 +1395,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J13" s="4" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1435,12 +1435,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1465,33 +1465,33 @@
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>R$ 38,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>6</v>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>▲ 200,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>16,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1508,12 +1508,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1538,7 +1538,7 @@
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>R$ 38,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
@@ -1547,24 +1547,24 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J15" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1581,12 +1581,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>18/05/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1620,7 +1620,7 @@
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
@@ -1654,12 +1654,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>18/05/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>07/06/2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1695,7 +1695,7 @@
       <c r="I17" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J17" s="4" t="inlineStr">
+      <c r="J17" s="3" t="inlineStr">
         <is>
           <t>▼ 100,0%</t>
         </is>
@@ -1727,12 +1727,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>07/06/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1766,7 +1766,7 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
@@ -1800,12 +1800,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1833,17 +1833,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I19" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1873,12 +1873,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>04/06/2026</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1903,7 +1903,7 @@
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 70,00</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
@@ -1912,24 +1912,24 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>5</v>
+      </c>
+      <c r="J20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>20,0%</t>
         </is>
       </c>
       <c r="L20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,8%</t>
         </is>
       </c>
       <c r="N20" s="2" t="inlineStr">
@@ -1946,12 +1946,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>04/06/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1979,17 +1979,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr">
@@ -2019,12 +2019,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2049,7 +2049,7 @@
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 35,00</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2058,24 +2058,24 @@
         </is>
       </c>
       <c r="I22" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J22" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>50,0%</t>
         </is>
       </c>
       <c r="L22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N22" s="2" t="inlineStr">
@@ -2092,12 +2092,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2131,11 +2131,11 @@
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J23" s="4" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K23" s="2" t="inlineStr">
@@ -2165,12 +2165,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2204,11 +2204,11 @@
         </is>
       </c>
       <c r="I24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J24" s="3" t="inlineStr">
         <is>
-          <t>▲ 100,0%</t>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K24" s="2" t="inlineStr">
@@ -2238,12 +2238,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2277,11 +2277,11 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" s="4" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+        <v>3</v>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
@@ -2311,12 +2311,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2344,17 +2344,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J26" s="3" t="inlineStr">
         <is>
-          <t>▲ 200,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2384,12 +2384,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 38,00</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2423,24 +2423,24 @@
         </is>
       </c>
       <c r="I27" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J27" s="4" t="inlineStr">
+        <is>
+          <t>▲ 150,0%</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>20,0%</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="4" t="inlineStr">
-        <is>
-          <t>▼ 50,0%</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -2457,12 +2457,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2490,17 +2490,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H28" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H28" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2530,12 +2530,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>26/05/2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2560,7 +2560,7 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>R$ 29,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
@@ -2569,11 +2569,11 @@
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="J29" s="4" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▲ 300,0%</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
@@ -2582,11 +2582,11 @@
         </is>
       </c>
       <c r="L29" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>0,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -2603,12 +2603,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>26/05/2026</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2636,17 +2636,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H30" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J30" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>1</v>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
@@ -2676,12 +2676,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2706,7 +2706,7 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>R$ 139,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
@@ -2717,22 +2717,22 @@
       <c r="I31" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J31" s="3" t="inlineStr">
+      <c r="J31" s="4" t="inlineStr">
         <is>
           <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
         <is>
-          <t>100,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L31" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>1,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N31" s="2" t="inlineStr">
@@ -2749,12 +2749,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2790,9 +2790,9 @@
       <c r="I32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2822,12 +2822,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2861,7 +2861,7 @@
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J33" s="2" t="inlineStr">
         <is>
@@ -2895,12 +2895,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2928,15 +2928,15 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H34" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I34" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J34" s="4" t="inlineStr">
+      <c r="J34" s="3" t="inlineStr">
         <is>
           <t>▼ 100,0%</t>
         </is>
@@ -2968,12 +2968,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -2998,33 +2998,33 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 38,00</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="I35" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J35" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>16,7%</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J35" s="4" t="inlineStr">
-        <is>
-          <t>▼ 50,0%</t>
-        </is>
-      </c>
-      <c r="K35" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L35" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N35" s="2" t="inlineStr">
@@ -3041,12 +3041,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3071,7 +3071,7 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 38,00</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
@@ -3084,20 +3084,20 @@
       </c>
       <c r="J36" s="4" t="inlineStr">
         <is>
-          <t>▼ 33,3%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>50,0%</t>
         </is>
       </c>
       <c r="L36" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N36" s="2" t="inlineStr">
@@ -3114,12 +3114,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>18/05/2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3153,11 +3153,11 @@
         </is>
       </c>
       <c r="I37" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J37" s="3" t="inlineStr">
-        <is>
-          <t>▲ 50,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3187,12 +3187,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>18/05/2026</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3220,17 +3220,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H38" s="4" t="inlineStr">
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
         <is>
           <t>▼ 100,0%</t>
-        </is>
-      </c>
-      <c r="I38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J38" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
@@ -3260,12 +3260,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>R$ 30,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3299,24 +3299,24 @@
         </is>
       </c>
       <c r="I39" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L39" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3333,12 +3333,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3372,11 +3372,11 @@
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+        <v>0</v>
+      </c>
+      <c r="J40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr">
@@ -3406,12 +3406,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3445,11 +3445,11 @@
         </is>
       </c>
       <c r="I41" s="2" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J41" s="3" t="inlineStr">
         <is>
-          <t>▲ 50,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K41" s="2" t="inlineStr">
@@ -3479,12 +3479,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3518,11 +3518,11 @@
         </is>
       </c>
       <c r="I42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J42" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K42" s="2" t="inlineStr">
@@ -3552,12 +3552,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3591,7 +3591,7 @@
         </is>
       </c>
       <c r="I43" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J43" s="2" t="inlineStr">
         <is>
@@ -3625,12 +3625,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3666,9 +3666,9 @@
       <c r="I44" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3698,12 +3698,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3737,11 +3737,11 @@
         </is>
       </c>
       <c r="I45" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J45" s="4" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -3771,12 +3771,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3812,9 +3812,9 @@
       <c r="I46" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J46" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K46" s="2" t="inlineStr">
@@ -3844,12 +3844,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3883,11 +3883,11 @@
         </is>
       </c>
       <c r="I47" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J47" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>3</v>
+      </c>
+      <c r="J47" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3917,12 +3917,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3956,11 +3956,11 @@
         </is>
       </c>
       <c r="I48" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -3990,12 +3990,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4023,17 +4023,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I49" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J49" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4063,12 +4063,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4093,7 +4093,7 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 29,00</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4102,24 +4102,24 @@
         </is>
       </c>
       <c r="I50" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K50" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L50" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J50" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K50" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L50" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,3%</t>
         </is>
       </c>
       <c r="N50" s="2" t="inlineStr">
@@ -4136,12 +4136,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4169,17 +4169,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H51" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I51" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J51" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4209,12 +4209,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4239,7 +4239,7 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 139,00</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -4248,24 +4248,24 @@
         </is>
       </c>
       <c r="I52" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J52" s="4" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>100,0%</t>
         </is>
       </c>
       <c r="L52" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,7%</t>
         </is>
       </c>
       <c r="N52" s="2" t="inlineStr">
@@ -4282,12 +4282,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4325,7 +4325,7 @@
       </c>
       <c r="J53" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -4355,12 +4355,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4394,11 +4394,11 @@
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J54" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J54" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -4428,12 +4428,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -4467,11 +4467,11 @@
         </is>
       </c>
       <c r="I55" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J55" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>0</v>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
@@ -4501,12 +4501,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -4542,9 +4542,9 @@
       <c r="I56" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J56" s="4" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -4574,12 +4574,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -4613,11 +4613,11 @@
         </is>
       </c>
       <c r="I57" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>2</v>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="K57" s="2" t="inlineStr">
@@ -4647,12 +4647,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4688,7 +4688,7 @@
       <c r="I58" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="J58" s="3" t="inlineStr">
+      <c r="J58" s="4" t="inlineStr">
         <is>
           <t>▲ 50,0%</t>
         </is>
@@ -4720,12 +4720,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4753,17 +4753,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H59" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I59" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+      <c r="J59" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
@@ -4793,12 +4793,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 30,00</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
@@ -4832,24 +4832,24 @@
         </is>
       </c>
       <c r="I60" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K60" s="2" t="inlineStr">
+        <is>
+          <t>50,0%</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N60" s="2" t="inlineStr">
@@ -4866,12 +4866,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -4905,11 +4905,11 @@
         </is>
       </c>
       <c r="I61" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -4939,12 +4939,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4978,11 +4978,11 @@
         </is>
       </c>
       <c r="I62" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J62" s="3" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>3</v>
+      </c>
+      <c r="J62" s="4" t="inlineStr">
+        <is>
+          <t>▲ 50,0%</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -5012,12 +5012,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -5051,11 +5051,11 @@
         </is>
       </c>
       <c r="I63" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J63" s="4" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
@@ -5085,78 +5085,1611 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
+          <t>22/04/2026</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I64" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J64" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K64" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M64" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N64" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>21/04/2026</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E65" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J65" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K65" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M65" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N65" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>20/04/2026</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K66" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M66" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N66" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O66" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>19/04/2026</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E67" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M67" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N67" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O67" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>18/04/2026</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J68" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K68" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M68" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N68" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>17/04/2026</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E69" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K69" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M69" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N69" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O69" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>16/04/2026</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I70" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J70" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K70" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L70" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M70" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N70" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O70" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>15/04/2026</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>14/04/2026</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E71" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I71" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J71" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K71" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L71" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M71" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N71" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O71" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>14/04/2026</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E72" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H72" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K72" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L72" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M72" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N72" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O72" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>13/04/2026</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E73" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H73" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K73" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L73" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M73" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N73" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O73" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E74" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H74" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I74" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J74" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K74" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L74" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M74" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N74" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>11/04/2026</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E75" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H75" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J75" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K75" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L75" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M75" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N75" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O75" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>10/04/2026</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E76" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H76" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I76" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J76" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K76" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L76" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M76" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N76" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>09/04/2026</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E77" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H77" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I77" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J77" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
+        </is>
+      </c>
+      <c r="K77" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L77" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M77" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N77" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O77" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>08/04/2026</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E78" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H78" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I78" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K78" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L78" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M78" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N78" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>07/04/2026</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>06/04/2026</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E79" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H79" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I79" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="J79" s="4" t="inlineStr">
+        <is>
+          <t>▲ 50,0%</t>
+        </is>
+      </c>
+      <c r="K79" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L79" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M79" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N79" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O79" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>06/04/2026</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J80" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
+        </is>
+      </c>
+      <c r="K80" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L80" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M80" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N80" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O80" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E81" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H81" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I81" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J81" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K81" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L81" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M81" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N81" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K82" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L82" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M82" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N82" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E83" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H83" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I83" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J83" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
+        </is>
+      </c>
+      <c r="K83" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L83" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M83" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N83" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
           <t>01/04/2026</t>
         </is>
       </c>
-      <c r="B64" s="2" t="inlineStr">
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I84" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
+        </is>
+      </c>
+      <c r="K84" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L84" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M84" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N84" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O84" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="C64" s="2" t="inlineStr">
-        <is>
-          <t>UTD-028-CZ</t>
-        </is>
-      </c>
-      <c r="D64" s="2" t="inlineStr">
-        <is>
-          <t>Organizador Tampa</t>
-        </is>
-      </c>
-      <c r="E64" s="2" t="inlineStr">
-        <is>
-          <t>4508101335</t>
-        </is>
-      </c>
-      <c r="F64" s="2" t="inlineStr">
-        <is>
-          <t>R$ 39,90</t>
-        </is>
-      </c>
-      <c r="G64" s="2" t="inlineStr">
-        <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I64" s="2" t="n">
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E85" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H85" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I85" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J64" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K64" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M64" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="N64" s="2" t="inlineStr">
-        <is>
-          <t>Sem calcular</t>
-        </is>
-      </c>
-      <c r="O64" s="2" t="inlineStr">
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K85" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L85" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M85" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N85" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O85" s="2" t="inlineStr">
         <is>
           <t>Boa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O64"/>
+  <autoFilter ref="A1:O85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
relatorios 26-27-28-29 mes junho
</commit_message>
<xml_diff>
--- a/saida_skus/SKU_UTD-028-CZ-ORGANIZADOR-TAMPA.xlsx
+++ b/saida_skus/SKU_UTD-028-CZ-ORGANIZADOR-TAMPA.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Analise" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$88</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Analise'!$A$1:$O$92</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -459,7 +459,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O88"/>
+  <dimension ref="A1:O92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -559,12 +559,12 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>26/06/2026</t>
+          <t>30/06/2026</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>29/06/2026</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -592,9 +592,9 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I2" s="2" t="n">
@@ -632,12 +632,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>25/06/2026</t>
+          <t>29/06/2026</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>24/06/2026</t>
+          <t>28/06/2026</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -662,7 +662,7 @@
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 34,00</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -680,15 +680,15 @@
       </c>
       <c r="K3" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>33,3%</t>
         </is>
       </c>
       <c r="L3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -705,12 +705,12 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>24/06/2026</t>
+          <t>28/06/2026</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -778,12 +778,12 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>23/06/2026</t>
+          <t>27/06/2026</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>26/06/2026</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -817,11 +817,11 @@
         </is>
       </c>
       <c r="I5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J5" s="3" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+        <v>3</v>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K5" s="2" t="inlineStr">
@@ -851,12 +851,12 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>22/06/2026</t>
+          <t>26/06/2026</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -884,17 +884,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H6" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I6" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>▼ 25,0%</t>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr">
@@ -924,12 +924,12 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>21/06/2026</t>
+          <t>25/06/2026</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026</t>
+          <t>24/06/2026</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -954,7 +954,7 @@
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>R$ 35,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
@@ -963,7 +963,7 @@
         </is>
       </c>
       <c r="I7" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
@@ -972,15 +972,15 @@
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>25,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -997,12 +997,12 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>20/06/2026</t>
+          <t>24/06/2026</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>19/06/2026</t>
+          <t>23/06/2026</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
@@ -1070,12 +1070,12 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>19/06/2026</t>
+          <t>23/06/2026</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
@@ -1111,9 +1111,9 @@
       <c r="I9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr">
@@ -1143,12 +1143,12 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>22/06/2026</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
@@ -1176,17 +1176,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I10" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>▼ 75,0%</t>
+          <t>▼ 25,0%</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
@@ -1216,12 +1216,12 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>17/06/2026</t>
+          <t>21/06/2026</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>16/06/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 35,00</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
@@ -1257,22 +1257,22 @@
       <c r="I11" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>▲ 300,0%</t>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>25,0%</t>
         </is>
       </c>
       <c r="L11" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1289,12 +1289,12 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>16/06/2026</t>
+          <t>20/06/2026</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>19/06/2026</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1328,11 +1328,11 @@
         </is>
       </c>
       <c r="I12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>▼ 75,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
@@ -1362,12 +1362,12 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>15/06/2026</t>
+          <t>19/06/2026</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>14/06/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
@@ -1401,11 +1401,11 @@
         </is>
       </c>
       <c r="I13" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J13" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
@@ -1435,12 +1435,12 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>14/06/2026</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026</t>
+          <t>17/06/2026</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1474,11 +1474,11 @@
         </is>
       </c>
       <c r="I14" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J14" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>1</v>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>▼ 75,0%</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
@@ -1508,12 +1508,12 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>13/06/2026</t>
+          <t>17/06/2026</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
@@ -1547,11 +1547,11 @@
         </is>
       </c>
       <c r="I15" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J15" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>4</v>
+      </c>
+      <c r="J15" s="4" t="inlineStr">
+        <is>
+          <t>▲ 300,0%</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
@@ -1581,12 +1581,12 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>12/06/2026</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
@@ -1620,11 +1620,11 @@
         </is>
       </c>
       <c r="I16" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>▼ 75,0%</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
@@ -1654,12 +1654,12 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>11/06/2026</t>
+          <t>15/06/2026</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>14/06/2026</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
@@ -1693,11 +1693,11 @@
         </is>
       </c>
       <c r="I17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>4</v>
+      </c>
+      <c r="J17" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K17" s="2" t="inlineStr">
@@ -1727,12 +1727,12 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>14/06/2026</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
@@ -1766,11 +1766,11 @@
         </is>
       </c>
       <c r="I18" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr">
@@ -1800,12 +1800,12 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026</t>
+          <t>12/06/2026</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
@@ -1839,11 +1839,11 @@
         </is>
       </c>
       <c r="I19" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr">
@@ -1873,12 +1873,12 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>08/06/2026</t>
+          <t>12/06/2026</t>
         </is>
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
@@ -1912,11 +1912,11 @@
         </is>
       </c>
       <c r="I20" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K20" s="2" t="inlineStr">
@@ -1946,12 +1946,12 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>07/06/2026</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
@@ -1985,7 +1985,7 @@
         </is>
       </c>
       <c r="I21" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
@@ -2019,12 +2019,12 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>06/06/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
@@ -2052,17 +2052,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H22" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I22" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K22" s="2" t="inlineStr">
@@ -2092,12 +2092,12 @@
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
         <is>
-          <t>05/06/2026</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
@@ -2122,7 +2122,7 @@
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>R$ 70,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2131,7 +2131,7 @@
         </is>
       </c>
       <c r="I23" s="2" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J23" s="2" t="inlineStr">
         <is>
@@ -2140,15 +2140,15 @@
       </c>
       <c r="K23" s="2" t="inlineStr">
         <is>
-          <t>20,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L23" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>0,8%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N23" s="2" t="inlineStr">
@@ -2165,12 +2165,12 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>04/06/2026</t>
+          <t>08/06/2026</t>
         </is>
       </c>
       <c r="B24" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026</t>
+          <t>07/06/2026</t>
         </is>
       </c>
       <c r="C24" s="2" t="inlineStr">
@@ -2198,9 +2198,9 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H24" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I24" s="2" t="n">
@@ -2238,12 +2238,12 @@
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
         <is>
-          <t>03/06/2026</t>
+          <t>07/06/2026</t>
         </is>
       </c>
       <c r="B25" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="C25" s="2" t="inlineStr">
@@ -2268,7 +2268,7 @@
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>R$ 35,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
@@ -2277,24 +2277,24 @@
         </is>
       </c>
       <c r="I25" s="2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L25" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N25" s="2" t="inlineStr">
@@ -2311,12 +2311,12 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>02/06/2026</t>
+          <t>06/06/2026</t>
         </is>
       </c>
       <c r="B26" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="C26" s="2" t="inlineStr">
@@ -2344,17 +2344,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I26" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K26" s="2" t="inlineStr">
@@ -2384,12 +2384,12 @@
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
         <is>
-          <t>01/06/2026</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="B27" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>04/06/2026</t>
         </is>
       </c>
       <c r="C27" s="2" t="inlineStr">
@@ -2414,7 +2414,7 @@
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 70,00</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2423,24 +2423,24 @@
         </is>
       </c>
       <c r="I27" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>20,0%</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J27" s="3" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
-        </is>
-      </c>
-      <c r="K27" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L27" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,8%</t>
         </is>
       </c>
       <c r="N27" s="2" t="inlineStr">
@@ -2457,12 +2457,12 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>31/05/2026</t>
+          <t>04/06/2026</t>
         </is>
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
@@ -2490,17 +2490,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I28" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K28" s="2" t="inlineStr">
@@ -2530,12 +2530,12 @@
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>30/05/2026</t>
+          <t>03/06/2026</t>
         </is>
       </c>
       <c r="B29" s="2" t="inlineStr">
         <is>
-          <t>29/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="C29" s="2" t="inlineStr">
@@ -2560,33 +2560,33 @@
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H29" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+          <t>R$ 35,00</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I29" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J29" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K29" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>50,0%</t>
         </is>
       </c>
       <c r="L29" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N29" s="2" t="inlineStr">
@@ -2603,12 +2603,12 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>29/05/2026</t>
+          <t>02/06/2026</t>
         </is>
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>28/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
@@ -2633,7 +2633,7 @@
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>R$ 38,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
@@ -2642,24 +2642,24 @@
         </is>
       </c>
       <c r="I30" s="2" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J30" s="4" t="inlineStr">
         <is>
-          <t>▲ 150,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K30" s="2" t="inlineStr">
         <is>
-          <t>20,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L30" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>0,6%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N30" s="2" t="inlineStr">
@@ -2676,12 +2676,12 @@
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
         <is>
-          <t>28/05/2026</t>
+          <t>01/06/2026</t>
         </is>
       </c>
       <c r="B31" s="2" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="C31" s="2" t="inlineStr">
@@ -2715,11 +2715,11 @@
         </is>
       </c>
       <c r="I31" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J31" s="3" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K31" s="2" t="inlineStr">
@@ -2749,12 +2749,12 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>27/05/2026</t>
+          <t>31/05/2026</t>
         </is>
       </c>
       <c r="B32" s="2" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="C32" s="2" t="inlineStr">
@@ -2788,11 +2788,11 @@
         </is>
       </c>
       <c r="I32" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>▲ 300,0%</t>
+        <v>3</v>
+      </c>
+      <c r="J32" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K32" s="2" t="inlineStr">
@@ -2822,12 +2822,12 @@
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
         <is>
-          <t>26/05/2026</t>
+          <t>30/05/2026</t>
         </is>
       </c>
       <c r="B33" s="2" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="C33" s="2" t="inlineStr">
@@ -2855,17 +2855,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H33" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I33" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J33" s="3" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K33" s="2" t="inlineStr">
@@ -2895,12 +2895,12 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>25/05/2026</t>
+          <t>29/05/2026</t>
         </is>
       </c>
       <c r="B34" s="2" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="C34" s="2" t="inlineStr">
@@ -2925,7 +2925,7 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 38,00</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
@@ -2934,24 +2934,24 @@
         </is>
       </c>
       <c r="I34" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J34" s="4" t="inlineStr">
         <is>
-          <t>▲ 100,0%</t>
+          <t>▲ 150,0%</t>
         </is>
       </c>
       <c r="K34" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>20,0%</t>
         </is>
       </c>
       <c r="L34" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,6%</t>
         </is>
       </c>
       <c r="N34" s="2" t="inlineStr">
@@ -2968,12 +2968,12 @@
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
         <is>
-          <t>24/05/2026</t>
+          <t>28/05/2026</t>
         </is>
       </c>
       <c r="B35" s="2" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="C35" s="2" t="inlineStr">
@@ -3007,7 +3007,7 @@
         </is>
       </c>
       <c r="I35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J35" s="3" t="inlineStr">
         <is>
@@ -3041,12 +3041,12 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>23/05/2026</t>
+          <t>27/05/2026</t>
         </is>
       </c>
       <c r="B36" s="2" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>26/05/2026</t>
         </is>
       </c>
       <c r="C36" s="2" t="inlineStr">
@@ -3080,11 +3080,11 @@
         </is>
       </c>
       <c r="I36" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>4</v>
+      </c>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>▲ 300,0%</t>
         </is>
       </c>
       <c r="K36" s="2" t="inlineStr">
@@ -3114,12 +3114,12 @@
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
         <is>
-          <t>22/05/2026</t>
+          <t>26/05/2026</t>
         </is>
       </c>
       <c r="B37" s="2" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="C37" s="2" t="inlineStr">
@@ -3147,17 +3147,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H37" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I37" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J37" s="3" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K37" s="2" t="inlineStr">
@@ -3187,12 +3187,12 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>21/05/2026</t>
+          <t>25/05/2026</t>
         </is>
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
@@ -3217,33 +3217,33 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>R$ 38,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="I38" s="2" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="J38" s="4" t="inlineStr">
         <is>
-          <t>▲ 200,0%</t>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr">
         <is>
-          <t>16,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L38" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>0,4%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N38" s="2" t="inlineStr">
@@ -3260,12 +3260,12 @@
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
         <is>
-          <t>20/05/2026</t>
+          <t>24/05/2026</t>
         </is>
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
@@ -3290,7 +3290,7 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>R$ 38,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3299,24 +3299,24 @@
         </is>
       </c>
       <c r="I39" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J39" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K39" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L39" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N39" s="2" t="inlineStr">
@@ -3333,12 +3333,12 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>19/05/2026</t>
+          <t>23/05/2026</t>
         </is>
       </c>
       <c r="B40" s="2" t="inlineStr">
         <is>
-          <t>18/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="C40" s="2" t="inlineStr">
@@ -3372,7 +3372,7 @@
         </is>
       </c>
       <c r="I40" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
@@ -3406,12 +3406,12 @@
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
         <is>
-          <t>18/05/2026</t>
+          <t>22/05/2026</t>
         </is>
       </c>
       <c r="B41" s="2" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="C41" s="2" t="inlineStr">
@@ -3439,9 +3439,9 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I41" s="2" t="n">
@@ -3479,12 +3479,12 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>17/05/2026</t>
+          <t>21/05/2026</t>
         </is>
       </c>
       <c r="B42" s="2" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="C42" s="2" t="inlineStr">
@@ -3509,33 +3509,33 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 38,00</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="I42" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
+        </is>
+      </c>
+      <c r="K42" s="2" t="inlineStr">
+        <is>
+          <t>16,7%</t>
+        </is>
+      </c>
+      <c r="L42" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,4%</t>
         </is>
       </c>
       <c r="N42" s="2" t="inlineStr">
@@ -3552,12 +3552,12 @@
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
         <is>
-          <t>16/05/2026</t>
+          <t>20/05/2026</t>
         </is>
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
@@ -3582,7 +3582,7 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 38,00</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3591,24 +3591,24 @@
         </is>
       </c>
       <c r="I43" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J43" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>2</v>
+      </c>
+      <c r="J43" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K43" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>50,0%</t>
         </is>
       </c>
       <c r="L43" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N43" s="2" t="inlineStr">
@@ -3625,12 +3625,12 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>15/05/2026</t>
+          <t>19/05/2026</t>
         </is>
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>18/05/2026</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
@@ -3664,11 +3664,11 @@
         </is>
       </c>
       <c r="I44" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J44" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K44" s="2" t="inlineStr">
@@ -3698,12 +3698,12 @@
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026</t>
+          <t>18/05/2026</t>
         </is>
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3737,11 +3737,11 @@
         </is>
       </c>
       <c r="I45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>0</v>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K45" s="2" t="inlineStr">
@@ -3771,12 +3771,12 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>13/05/2026</t>
+          <t>17/05/2026</t>
         </is>
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
@@ -3810,7 +3810,7 @@
         </is>
       </c>
       <c r="I46" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J46" s="2" t="inlineStr">
         <is>
@@ -3844,12 +3844,12 @@
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
         <is>
-          <t>12/05/2026</t>
+          <t>16/05/2026</t>
         </is>
       </c>
       <c r="B47" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="C47" s="2" t="inlineStr">
@@ -3885,9 +3885,9 @@
       <c r="I47" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J47" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K47" s="2" t="inlineStr">
@@ -3917,12 +3917,12 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>15/05/2026</t>
         </is>
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
@@ -3956,11 +3956,11 @@
         </is>
       </c>
       <c r="I48" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J48" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K48" s="2" t="inlineStr">
@@ -3990,12 +3990,12 @@
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
         <is>
-          <t>10/05/2026</t>
+          <t>14/05/2026</t>
         </is>
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
@@ -4031,9 +4031,9 @@
       <c r="I49" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J49" s="3" t="inlineStr">
-        <is>
-          <t>▼ 66,7%</t>
+      <c r="J49" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K49" s="2" t="inlineStr">
@@ -4063,12 +4063,12 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>09/05/2026</t>
+          <t>13/05/2026</t>
         </is>
       </c>
       <c r="B50" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="C50" s="2" t="inlineStr">
@@ -4102,11 +4102,11 @@
         </is>
       </c>
       <c r="I50" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J50" s="4" t="inlineStr">
-        <is>
-          <t>▲ 200,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J50" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K50" s="2" t="inlineStr">
@@ -4136,12 +4136,12 @@
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
         <is>
-          <t>08/05/2026</t>
+          <t>12/05/2026</t>
         </is>
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
@@ -4175,11 +4175,11 @@
         </is>
       </c>
       <c r="I51" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J51" s="3" t="inlineStr">
         <is>
-          <t>▼ 50,0%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K51" s="2" t="inlineStr">
@@ -4209,12 +4209,12 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>07/05/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
@@ -4242,17 +4242,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H52" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I52" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J52" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K52" s="2" t="inlineStr">
@@ -4282,12 +4282,12 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>06/05/2026</t>
+          <t>10/05/2026</t>
         </is>
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
@@ -4312,7 +4312,7 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>R$ 29,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4321,11 +4321,11 @@
         </is>
       </c>
       <c r="I53" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J53" s="3" t="inlineStr">
         <is>
-          <t>▼ 100,0%</t>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K53" s="2" t="inlineStr">
@@ -4334,11 +4334,11 @@
         </is>
       </c>
       <c r="L53" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>0,3%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N53" s="2" t="inlineStr">
@@ -4355,12 +4355,12 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>05/05/2026</t>
+          <t>09/05/2026</t>
         </is>
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
@@ -4388,17 +4388,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H54" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="I54" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>3</v>
+      </c>
+      <c r="J54" s="4" t="inlineStr">
+        <is>
+          <t>▲ 200,0%</t>
         </is>
       </c>
       <c r="K54" s="2" t="inlineStr">
@@ -4428,12 +4428,12 @@
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
         <is>
-          <t>04/05/2026</t>
+          <t>08/05/2026</t>
         </is>
       </c>
       <c r="B55" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="C55" s="2" t="inlineStr">
@@ -4458,7 +4458,7 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>R$ 139,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
@@ -4467,24 +4467,24 @@
         </is>
       </c>
       <c r="I55" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J55" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K55" s="2" t="inlineStr">
         <is>
-          <t>100,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L55" s="2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>1,7%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N55" s="2" t="inlineStr">
@@ -4501,12 +4501,12 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>03/05/2026</t>
+          <t>07/05/2026</t>
         </is>
       </c>
       <c r="B56" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="C56" s="2" t="inlineStr">
@@ -4534,17 +4534,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H56" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I56" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J56" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K56" s="2" t="inlineStr">
@@ -4574,12 +4574,12 @@
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>02/05/2026</t>
+          <t>06/05/2026</t>
         </is>
       </c>
       <c r="B57" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="C57" s="2" t="inlineStr">
@@ -4604,7 +4604,7 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 29,00</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
@@ -4613,24 +4613,24 @@
         </is>
       </c>
       <c r="I57" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K57" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L57" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L57" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,3%</t>
         </is>
       </c>
       <c r="N57" s="2" t="inlineStr">
@@ -4647,12 +4647,12 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>01/05/2026</t>
+          <t>05/05/2026</t>
         </is>
       </c>
       <c r="B58" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="C58" s="2" t="inlineStr">
@@ -4680,17 +4680,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I58" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J58" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K58" s="2" t="inlineStr">
@@ -4720,12 +4720,12 @@
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
         <is>
-          <t>30/04/2026</t>
+          <t>04/05/2026</t>
         </is>
       </c>
       <c r="B59" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="C59" s="2" t="inlineStr">
@@ -4750,7 +4750,7 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 139,00</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
@@ -4759,24 +4759,24 @@
         </is>
       </c>
       <c r="I59" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J59" s="3" t="inlineStr">
-        <is>
-          <t>▼ 50,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J59" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K59" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>100,0%</t>
         </is>
       </c>
       <c r="L59" s="2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>1,7%</t>
         </is>
       </c>
       <c r="N59" s="2" t="inlineStr">
@@ -4793,12 +4793,12 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>29/04/2026</t>
+          <t>03/05/2026</t>
         </is>
       </c>
       <c r="B60" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="C60" s="2" t="inlineStr">
@@ -4832,11 +4832,11 @@
         </is>
       </c>
       <c r="I60" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J60" s="3" t="inlineStr">
-        <is>
-          <t>▼ 33,3%</t>
+        <v>1</v>
+      </c>
+      <c r="J60" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K60" s="2" t="inlineStr">
@@ -4866,12 +4866,12 @@
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
         <is>
-          <t>28/04/2026</t>
+          <t>02/05/2026</t>
         </is>
       </c>
       <c r="B61" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="C61" s="2" t="inlineStr">
@@ -4905,11 +4905,11 @@
         </is>
       </c>
       <c r="I61" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J61" s="4" t="inlineStr">
-        <is>
-          <t>▲ 50,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J61" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K61" s="2" t="inlineStr">
@@ -4939,12 +4939,12 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>27/04/2026</t>
+          <t>01/05/2026</t>
         </is>
       </c>
       <c r="B62" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="C62" s="2" t="inlineStr">
@@ -4972,17 +4972,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H62" s="3" t="inlineStr">
+      <c r="H62" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I62" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
         <is>
           <t>▼ 100,0%</t>
-        </is>
-      </c>
-      <c r="I62" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
         </is>
       </c>
       <c r="K62" s="2" t="inlineStr">
@@ -5012,12 +5012,12 @@
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
         <is>
-          <t>26/04/2026</t>
+          <t>30/04/2026</t>
         </is>
       </c>
       <c r="B63" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="C63" s="2" t="inlineStr">
@@ -5042,7 +5042,7 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>R$ 30,00</t>
+          <t>R$ 0,00</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
@@ -5051,24 +5051,24 @@
         </is>
       </c>
       <c r="I63" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J63" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>1</v>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
         </is>
       </c>
       <c r="K63" s="2" t="inlineStr">
         <is>
-          <t>50,0%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="L63" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>0,5%</t>
+          <t>0,0%</t>
         </is>
       </c>
       <c r="N63" s="2" t="inlineStr">
@@ -5085,12 +5085,12 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>25/04/2026</t>
+          <t>29/04/2026</t>
         </is>
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="C64" s="2" t="inlineStr">
@@ -5158,12 +5158,12 @@
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
         <is>
-          <t>24/04/2026</t>
+          <t>28/04/2026</t>
         </is>
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="C65" s="2" t="inlineStr">
@@ -5231,12 +5231,12 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>23/04/2026</t>
+          <t>27/04/2026</t>
         </is>
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="C66" s="2" t="inlineStr">
@@ -5264,17 +5264,17 @@
           <t>R$ 0,00</t>
         </is>
       </c>
-      <c r="H66" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="I66" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J66" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+      <c r="J66" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K66" s="2" t="inlineStr">
@@ -5304,12 +5304,12 @@
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
         <is>
-          <t>22/04/2026</t>
+          <t>26/04/2026</t>
         </is>
       </c>
       <c r="B67" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="C67" s="2" t="inlineStr">
@@ -5334,7 +5334,7 @@
       </c>
       <c r="G67" s="2" t="inlineStr">
         <is>
-          <t>R$ 0,00</t>
+          <t>R$ 30,00</t>
         </is>
       </c>
       <c r="H67" s="2" t="inlineStr">
@@ -5343,24 +5343,24 @@
         </is>
       </c>
       <c r="I67" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J67" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
+        </is>
+      </c>
+      <c r="K67" s="2" t="inlineStr">
+        <is>
+          <t>50,0%</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J67" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K67" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L67" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>0,0%</t>
+          <t>0,5%</t>
         </is>
       </c>
       <c r="N67" s="2" t="inlineStr">
@@ -5377,12 +5377,12 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>21/04/2026</t>
+          <t>25/04/2026</t>
         </is>
       </c>
       <c r="B68" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="C68" s="2" t="inlineStr">
@@ -5416,11 +5416,11 @@
         </is>
       </c>
       <c r="I68" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J68" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>2</v>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>▼ 33,3%</t>
         </is>
       </c>
       <c r="K68" s="2" t="inlineStr">
@@ -5450,12 +5450,12 @@
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
         <is>
-          <t>20/04/2026</t>
+          <t>24/04/2026</t>
         </is>
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
@@ -5489,11 +5489,11 @@
         </is>
       </c>
       <c r="I69" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J69" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>3</v>
+      </c>
+      <c r="J69" s="4" t="inlineStr">
+        <is>
+          <t>▲ 50,0%</t>
         </is>
       </c>
       <c r="K69" s="2" t="inlineStr">
@@ -5523,12 +5523,12 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>19/04/2026</t>
+          <t>23/04/2026</t>
         </is>
       </c>
       <c r="B70" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="C70" s="2" t="inlineStr">
@@ -5562,11 +5562,11 @@
         </is>
       </c>
       <c r="I70" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J70" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+        <v>2</v>
+      </c>
+      <c r="J70" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K70" s="2" t="inlineStr">
@@ -5596,12 +5596,12 @@
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
         <is>
-          <t>18/04/2026</t>
+          <t>22/04/2026</t>
         </is>
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="C71" s="2" t="inlineStr">
@@ -5635,7 +5635,7 @@
         </is>
       </c>
       <c r="I71" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J71" s="2" t="inlineStr">
         <is>
@@ -5669,12 +5669,12 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>17/04/2026</t>
+          <t>21/04/2026</t>
         </is>
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="C72" s="2" t="inlineStr">
@@ -5710,9 +5710,9 @@
       <c r="I72" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="J72" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+      <c r="J72" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K72" s="2" t="inlineStr">
@@ -5742,12 +5742,12 @@
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
         <is>
-          <t>16/04/2026</t>
+          <t>20/04/2026</t>
         </is>
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="C73" s="2" t="inlineStr">
@@ -5781,11 +5781,11 @@
         </is>
       </c>
       <c r="I73" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>0%</t>
+        <v>0</v>
+      </c>
+      <c r="J73" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K73" s="2" t="inlineStr">
@@ -5815,12 +5815,12 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>15/04/2026</t>
+          <t>19/04/2026</t>
         </is>
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
@@ -5888,12 +5888,12 @@
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
         <is>
-          <t>14/04/2026</t>
+          <t>18/04/2026</t>
         </is>
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="C75" s="2" t="inlineStr">
@@ -5961,12 +5961,12 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>13/04/2026</t>
+          <t>17/04/2026</t>
         </is>
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="C76" s="2" t="inlineStr">
@@ -6034,12 +6034,12 @@
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>16/04/2026</t>
         </is>
       </c>
       <c r="B77" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="C77" s="2" t="inlineStr">
@@ -6077,7 +6077,7 @@
       </c>
       <c r="J77" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>0%</t>
         </is>
       </c>
       <c r="K77" s="2" t="inlineStr">
@@ -6107,12 +6107,12 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>11/04/2026</t>
+          <t>15/04/2026</t>
         </is>
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="C78" s="2" t="inlineStr">
@@ -6146,11 +6146,11 @@
         </is>
       </c>
       <c r="I78" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J78" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J78" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="K78" s="2" t="inlineStr">
@@ -6180,12 +6180,12 @@
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
         <is>
-          <t>10/04/2026</t>
+          <t>14/04/2026</t>
         </is>
       </c>
       <c r="B79" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="C79" s="2" t="inlineStr">
@@ -6219,11 +6219,11 @@
         </is>
       </c>
       <c r="I79" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J79" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K79" s="2" t="inlineStr">
@@ -6253,12 +6253,12 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>09/04/2026</t>
+          <t>13/04/2026</t>
         </is>
       </c>
       <c r="B80" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C80" s="2" t="inlineStr">
@@ -6292,11 +6292,11 @@
         </is>
       </c>
       <c r="I80" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>▼ 66,7%</t>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K80" s="2" t="inlineStr">
@@ -6326,12 +6326,12 @@
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
         <is>
-          <t>08/04/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="B81" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="C81" s="2" t="inlineStr">
@@ -6365,11 +6365,11 @@
         </is>
       </c>
       <c r="I81" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J81" s="2" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K81" s="2" t="inlineStr">
@@ -6399,12 +6399,12 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>07/04/2026</t>
+          <t>11/04/2026</t>
         </is>
       </c>
       <c r="B82" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="C82" s="2" t="inlineStr">
@@ -6438,11 +6438,11 @@
         </is>
       </c>
       <c r="I82" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="J82" s="4" t="inlineStr">
-        <is>
-          <t>▲ 50,0%</t>
+        <v>0</v>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
         </is>
       </c>
       <c r="K82" s="2" t="inlineStr">
@@ -6472,12 +6472,12 @@
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
         <is>
-          <t>06/04/2026</t>
+          <t>10/04/2026</t>
         </is>
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="C83" s="2" t="inlineStr">
@@ -6511,11 +6511,11 @@
         </is>
       </c>
       <c r="I83" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="J83" s="4" t="inlineStr">
-        <is>
-          <t>▲ 100,0%</t>
+        <v>1</v>
+      </c>
+      <c r="J83" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K83" s="2" t="inlineStr">
@@ -6545,12 +6545,12 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>05/04/2026</t>
+          <t>09/04/2026</t>
         </is>
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="C84" s="2" t="inlineStr">
@@ -6586,9 +6586,9 @@
       <c r="I84" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="J84" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>▼ 66,7%</t>
         </is>
       </c>
       <c r="K84" s="2" t="inlineStr">
@@ -6618,12 +6618,12 @@
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
         <is>
-          <t>04/04/2026</t>
+          <t>08/04/2026</t>
         </is>
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="C85" s="2" t="inlineStr">
@@ -6657,11 +6657,11 @@
         </is>
       </c>
       <c r="I85" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="J85" s="3" t="inlineStr">
-        <is>
-          <t>▼ 100,0%</t>
+        <v>3</v>
+      </c>
+      <c r="J85" s="2" t="inlineStr">
+        <is>
+          <t>0%</t>
         </is>
       </c>
       <c r="K85" s="2" t="inlineStr">
@@ -6691,12 +6691,12 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>03/04/2026</t>
+          <t>07/04/2026</t>
         </is>
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="C86" s="2" t="inlineStr">
@@ -6730,11 +6730,11 @@
         </is>
       </c>
       <c r="I86" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J86" s="4" t="inlineStr">
         <is>
-          <t>▲ 100,0%</t>
+          <t>▲ 50,0%</t>
         </is>
       </c>
       <c r="K86" s="2" t="inlineStr">
@@ -6764,12 +6764,12 @@
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
         <is>
-          <t>02/04/2026</t>
+          <t>06/04/2026</t>
         </is>
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>01/04/2026</t>
+          <t>05/04/2026</t>
         </is>
       </c>
       <c r="C87" s="2" t="inlineStr">
@@ -6803,11 +6803,11 @@
         </is>
       </c>
       <c r="I87" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="J87" s="3" t="inlineStr">
-        <is>
-          <t>▼ 50,0%</t>
+        <v>2</v>
+      </c>
+      <c r="J87" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
         </is>
       </c>
       <c r="K87" s="2" t="inlineStr">
@@ -6837,78 +6837,370 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
+          <t>05/04/2026</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I88" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L88" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>04/04/2026</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E89" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H89" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J89" s="3" t="inlineStr">
+        <is>
+          <t>▼ 100,0%</t>
+        </is>
+      </c>
+      <c r="K89" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L89" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M89" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N89" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O89" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>03/04/2026</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I90" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="J90" s="4" t="inlineStr">
+        <is>
+          <t>▲ 100,0%</t>
+        </is>
+      </c>
+      <c r="K90" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L90" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M90" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N90" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>02/04/2026</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
           <t>01/04/2026</t>
         </is>
       </c>
-      <c r="B88" s="2" t="inlineStr">
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E91" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H91" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I91" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J91" s="3" t="inlineStr">
+        <is>
+          <t>▼ 50,0%</t>
+        </is>
+      </c>
+      <c r="K91" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L91" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M91" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N91" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O91" s="2" t="inlineStr">
+        <is>
+          <t>Boa</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>01/04/2026</t>
+        </is>
+      </c>
+      <c r="B92" s="2" t="inlineStr">
         <is>
           <t>31/03/2026</t>
         </is>
       </c>
-      <c r="C88" s="2" t="inlineStr">
-        <is>
-          <t>UTD-028-CZ</t>
-        </is>
-      </c>
-      <c r="D88" s="2" t="inlineStr">
-        <is>
-          <t>Organizador Tampa</t>
-        </is>
-      </c>
-      <c r="E88" s="2" t="inlineStr">
-        <is>
-          <t>4508101335</t>
-        </is>
-      </c>
-      <c r="F88" s="2" t="inlineStr">
-        <is>
-          <t>R$ 39,90</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr">
-        <is>
-          <t>R$ 0,00</t>
-        </is>
-      </c>
-      <c r="H88" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="n">
+      <c r="C92" s="2" t="inlineStr">
+        <is>
+          <t>UTD-028-CZ</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Organizador Tampa</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>4508101335</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>R$ 39,90</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>R$ 0,00</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I92" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="J88" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K88" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="L88" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="M88" s="2" t="inlineStr">
-        <is>
-          <t>0,0%</t>
-        </is>
-      </c>
-      <c r="N88" s="2" t="inlineStr">
-        <is>
-          <t>Sem calcular</t>
-        </is>
-      </c>
-      <c r="O88" s="2" t="inlineStr">
+      <c r="J92" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K92" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="L92" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M92" s="2" t="inlineStr">
+        <is>
+          <t>0,0%</t>
+        </is>
+      </c>
+      <c r="N92" s="2" t="inlineStr">
+        <is>
+          <t>Sem calcular</t>
+        </is>
+      </c>
+      <c r="O92" s="2" t="inlineStr">
         <is>
           <t>Boa</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O88"/>
+  <autoFilter ref="A1:O92"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>